<commit_message>
Refactor output directory structure: migrate comparisons and text comparisons to resultats
- Updated all relevant scripts and modules to reflect the new output path for comparisons.
- Introduced a new script to migrate existing comparison files from the old structure to the new one.
- Adjusted documentation and comments to align with the new output organization.
- Added a full pipeline script to orchestrate the execution of both indicator and text pipelines, consolidating results in the new output directory.
</commit_message>
<xml_diff>
--- a/outputs/resultats/td/2026_t1_vs_2025_t3/comparison.xlsx
+++ b/outputs/resultats/td/2026_t1_vs_2025_t3/comparison.xlsx
@@ -2005,7 +2005,9 @@
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>(1) Le changement est pertinent car il implique la suppression d'un tableau entier lié à la gestion du capital ; (2) Cela peut affecter la transparence et la compréhension des expositions nettes par région et contrepartie, ce qui est crucial pour l'évaluation des risques géographiques ; (3) Il s'agit d'une suppression structurelle qui pourrait indiquer un changement dans la manière dont la banque gère ou divulgue ses expositions.</t>
+          <t>Le changement constaté concerne la suppression d'un tableau intitulé 'TOTAL DE L’EXPOSITION NETTE PAR RÉGION ET CONTREPARTIE' dans la section de gestion du capital. Ce tableau fournissait des informations détaillées sur l'exposition nette de la banque par région, incluant des régions spécifiques comme l'Europe, le Royaume-Uni, l'Asie, et d'autres. La suppression de ce tableau peut indiquer un changement dans la manière dont la banque divulgue ses expositions régionales, ce qui pourrait avoir des implications sur la transparence des risques géographiques et la gestion du capital.
+D'un point de vue réglementaire, la divulgation des expositions par région est souvent requise pour évaluer le risque géographique et la concentration des actifs. La suppression de ce tableau pourrait affecter la capacité des régulateurs et des parties prenantes à évaluer correctement ces risques. Cela pourrait également avoir un impact sur la conformité avec les exigences de divulgation du Pilier 3 de Bâle III, qui vise à promouvoir la transparence et la discipline de marché.
+Il est recommandé d'investiguer ce changement pour comprendre les raisons derrière la suppression de ce tableau. Il pourrait s'agi</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Update comparison.xlsx with new data for 2026 T1 vs 2025 T3 analysis
</commit_message>
<xml_diff>
--- a/outputs/resultats/td/2026_t1_vs_2025_t3/comparison.xlsx
+++ b/outputs/resultats/td/2026_t1_vs_2025_t3/comparison.xlsx
@@ -2005,9 +2005,9 @@
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Le changement constaté concerne la suppression d'un tableau intitulé 'TOTAL DE L’EXPOSITION NETTE PAR RÉGION ET CONTREPARTIE' dans la section de gestion du capital. Ce tableau fournissait des informations détaillées sur l'exposition nette de la banque par région, incluant des régions spécifiques comme l'Europe, le Royaume-Uni, l'Asie, et d'autres. La suppression de ce tableau peut indiquer un changement dans la manière dont la banque divulgue ses expositions régionales, ce qui pourrait avoir des implications sur la transparence des risques géographiques et la gestion du capital.
-D'un point de vue réglementaire, la divulgation des expositions par région est souvent requise pour évaluer le risque géographique et la concentration des actifs. La suppression de ce tableau pourrait affecter la capacité des régulateurs et des parties prenantes à évaluer correctement ces risques. Cela pourrait également avoir un impact sur la conformité avec les exigences de divulgation du Pilier 3 de Bâle III, qui vise à promouvoir la transparence et la discipline de marché.
-Il est recommandé d'investiguer ce changement pour comprendre les raisons derrière la suppression de ce tableau. Il pourrait s'agi</t>
+          <t>Le changement constaté concerne la suppression d'un tableau intitulé 'TOTAL DE L’EXPOSITION NETTE PAR RÉGION ET CONTREPARTIE' dans la section de gestion du capital. Ce tableau fournissait des informations détaillées sur l'exposition nette de la banque par région, incluant des régions spécifiques comme l'Europe, le Royaume-Uni, l'Asie, et d'autres. La suppression de ce tableau peut indiquer un changement dans la manière dont la banque divulgue ses expositions géographiques, ce qui pourrait avoir des implications sur la transparence et la gestion des risques géographiques.
+D'un point de vue réglementaire, la divulgation des expositions par région est souvent requise pour évaluer la concentration des risques et la diversification géographique, ce qui est crucial pour le respect des exigences de Bâle III en matière de gestion des risques. La suppression de ce tableau pourrait signifier un changement dans la stratégie de divulgation ou une révision des méthodes de calcul des expositions, ce qui nécessite une attention particulière pour s'assurer que la banque reste conforme aux attentes réglementaires.
+Il est recommandé d'investiguer ce changement pour comprendre les raisons derrière</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">

</xml_diff>